<commit_message>
Consolidate into single master Shopify import CSV (WinBachat_Products_Shopify_Import.csv) and remove fragmented files
</commit_message>
<xml_diff>
--- a/WinBachat_New_Batches_Review_and_Audit.xlsx
+++ b/WinBachat_New_Batches_Review_and_Audit.xlsx
@@ -570,10 +570,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Comprehensive verification of Westpoint Electronics (282 items) &amp; MTS Gardening (170 items)</t>
-        </is>
-      </c>
-    </row>
+          <t>Single Unified Import: Westpoint Electronics (282 items) &amp; MTS Gardening (170 items)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -650,10 +651,10 @@
         <v>170</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
@@ -665,7 +666,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>23 duplicate listings drafted due to identical photos &amp; price conflicts</t>
+          <t>26 duplicate listings drafted due to identical photos &amp; price conflicts</t>
         </is>
       </c>
     </row>
@@ -679,10 +680,10 @@
         <v>452</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
@@ -694,10 +695,11 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>All 452 products ready in import sheets</t>
-        </is>
-      </c>
-    </row>
+          <t>ALL 452 PRODUCTS UNIFIED IN ONE SHOPIFY CSV</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
@@ -744,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1313,37 +1315,37 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Knock Down Bed Bug &amp; Flea Killer 100ml – Fenthion 35% EC</t>
+          <t>Bromoxynil MCPA Herbicide 100ml – Broadleaf Weed Control</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-100</t>
+          <t>MRT-WB-MTSGARDNING-033</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Pest Control &gt; Bed Bug Control</t>
+          <t>Gardening &gt; Gardening Fertilizers</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>1047.625</v>
+        <v>554.625</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-113</t>
+          <t>MRT-WB-MTSGARDNING-060</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Pest Control &gt; General Insects</t>
+          <t>Gardening &gt; Plants Insecticide/Fungicide</t>
         </is>
       </c>
       <c r="H12" s="11" t="n">
-        <v>1047.625</v>
+        <v>3451</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0</v>
+        <v>2896.375</v>
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
@@ -1362,12 +1364,12 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Knock Down Bed Bug &amp; Flea Killer 250ml – Fenthion 35% EC</t>
+          <t>Knock Down Bed Bug &amp; Flea Killer 100ml – Fenthion 35% EC</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-101</t>
+          <t>MRT-WB-MTSGARDNING-100</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -1376,11 +1378,11 @@
         </is>
       </c>
       <c r="E13" s="11" t="n">
-        <v>554.625</v>
+        <v>1047.625</v>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-114</t>
+          <t>MRT-WB-MTSGARDNING-113</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -1389,7 +1391,7 @@
         </is>
       </c>
       <c r="H13" s="11" t="n">
-        <v>554.625</v>
+        <v>1047.625</v>
       </c>
       <c r="I13" s="11" t="n">
         <v>0</v>
@@ -1411,12 +1413,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Knock Down Bed Bug &amp; Flea Killer 500ml – Fenthion 35% EC</t>
+          <t>Knock Down Bed Bug &amp; Flea Killer 250ml – Fenthion 35% EC</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-102</t>
+          <t>MRT-WB-MTSGARDNING-101</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -1425,11 +1427,11 @@
         </is>
       </c>
       <c r="E14" s="11" t="n">
-        <v>1109.25</v>
+        <v>554.625</v>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-115</t>
+          <t>MRT-WB-MTSGARDNING-114</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -1438,7 +1440,7 @@
         </is>
       </c>
       <c r="H14" s="11" t="n">
-        <v>1109.25</v>
+        <v>554.625</v>
       </c>
       <c r="I14" s="11" t="n">
         <v>0</v>
@@ -1460,12 +1462,12 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Knock Down Bed Bug &amp; Flea Killer 1000ml – Fenthion 35% EC</t>
+          <t>Knock Down Bed Bug &amp; Flea Killer 500ml – Fenthion 35% EC</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-103</t>
+          <t>MRT-WB-MTSGARDNING-102</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -1474,11 +1476,11 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>1972</v>
+        <v>1109.25</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-116</t>
+          <t>MRT-WB-MTSGARDNING-115</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
@@ -1487,7 +1489,7 @@
         </is>
       </c>
       <c r="H15" s="11" t="n">
-        <v>1972</v>
+        <v>1109.25</v>
       </c>
       <c r="I15" s="11" t="n">
         <v>0</v>
@@ -1509,25 +1511,25 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>One Shot DDVP EC 60 Insect Control Solution 100ml</t>
+          <t>Knock Down Bed Bug &amp; Flea Killer 1000ml – Fenthion 35% EC</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-085</t>
+          <t>MRT-WB-MTSGARDNING-103</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Pest Control &gt; Roaches Control</t>
+          <t>Pest Control &gt; Bed Bug Control</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>554.625</v>
+        <v>1972</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-121</t>
+          <t>MRT-WB-MTSGARDNING-116</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -1536,14 +1538,14 @@
         </is>
       </c>
       <c r="H16" s="11" t="n">
-        <v>3451</v>
+        <v>1972</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>2896.375</v>
+        <v>0</v>
       </c>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t>Identical photos (4 files)</t>
+          <t>Identical photos (2 files)</t>
         </is>
       </c>
       <c r="K16" s="10" t="inlineStr">
@@ -1558,12 +1560,12 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>One Shot DDVP EC 60 Insect Control Solution 250ml</t>
+          <t>One Shot DDVP EC 60 Insect Control Solution 100ml</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-086</t>
+          <t>MRT-WB-MTSGARDNING-085</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -1576,7 +1578,7 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-122</t>
+          <t>MRT-WB-MTSGARDNING-121</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -1585,10 +1587,10 @@
         </is>
       </c>
       <c r="H17" s="11" t="n">
-        <v>554.625</v>
+        <v>3451</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0</v>
+        <v>2896.375</v>
       </c>
       <c r="J17" s="10" t="inlineStr">
         <is>
@@ -1607,12 +1609,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>One Shot DDVP EC 60 Insect Control Solution 500ml</t>
+          <t>One Shot DDVP EC 60 Insect Control Solution 250ml</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-087</t>
+          <t>MRT-WB-MTSGARDNING-086</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -1621,11 +1623,11 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>1109.25</v>
+        <v>554.625</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-123</t>
+          <t>MRT-WB-MTSGARDNING-122</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -1634,7 +1636,7 @@
         </is>
       </c>
       <c r="H18" s="11" t="n">
-        <v>1109.25</v>
+        <v>554.625</v>
       </c>
       <c r="I18" s="11" t="n">
         <v>0</v>
@@ -1656,12 +1658,12 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>One Shot DDVP EC 60 Insect Control Solution 1000ml</t>
+          <t>One Shot DDVP EC 60 Insect Control Solution 500ml</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-088</t>
+          <t>MRT-WB-MTSGARDNING-087</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -1670,11 +1672,11 @@
         </is>
       </c>
       <c r="E19" s="11" t="n">
-        <v>1972</v>
+        <v>1109.25</v>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-124</t>
+          <t>MRT-WB-MTSGARDNING-123</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -1683,7 +1685,7 @@
         </is>
       </c>
       <c r="H19" s="11" t="n">
-        <v>1972</v>
+        <v>1109.25</v>
       </c>
       <c r="I19" s="11" t="n">
         <v>0</v>
@@ -1705,12 +1707,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Zero In Turbo Stream Permethrin 2.5 EC Pest Control 100ml</t>
+          <t>One Shot DDVP EC 60 Insect Control Solution 1000ml</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-089</t>
+          <t>MRT-WB-MTSGARDNING-088</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -1719,11 +1721,11 @@
         </is>
       </c>
       <c r="E20" s="11" t="n">
-        <v>3451</v>
+        <v>1972</v>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-125</t>
+          <t>MRT-WB-MTSGARDNING-124</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -1732,14 +1734,14 @@
         </is>
       </c>
       <c r="H20" s="11" t="n">
-        <v>3451</v>
+        <v>1972</v>
       </c>
       <c r="I20" s="11" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="10" t="inlineStr">
         <is>
-          <t>Identical photos (2 files)</t>
+          <t>Identical photos (4 files)</t>
         </is>
       </c>
       <c r="K20" s="10" t="inlineStr">
@@ -1754,12 +1756,12 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Zero In Turbo Stream Permethrin 2.5 EC Pest Control 250ml</t>
+          <t>Zero In Turbo Stream Permethrin 2.5 EC Pest Control 100ml</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-090</t>
+          <t>MRT-WB-MTSGARDNING-089</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
@@ -1768,11 +1770,11 @@
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>554.625</v>
+        <v>3451</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-126</t>
+          <t>MRT-WB-MTSGARDNING-125</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -1781,7 +1783,7 @@
         </is>
       </c>
       <c r="H21" s="11" t="n">
-        <v>554.625</v>
+        <v>3451</v>
       </c>
       <c r="I21" s="11" t="n">
         <v>0</v>
@@ -1803,12 +1805,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Zero In Turbo Stream Pest Control 500ml – Permethrin 2.5 EC</t>
+          <t>Zero In Turbo Stream Permethrin 2.5 EC Pest Control 250ml</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-091</t>
+          <t>MRT-WB-MTSGARDNING-090</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
@@ -1817,11 +1819,11 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>1109.25</v>
+        <v>554.625</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-127</t>
+          <t>MRT-WB-MTSGARDNING-126</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -1830,7 +1832,7 @@
         </is>
       </c>
       <c r="H22" s="11" t="n">
-        <v>1109.25</v>
+        <v>554.625</v>
       </c>
       <c r="I22" s="11" t="n">
         <v>0</v>
@@ -1852,12 +1854,12 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Zero In Turbo Stream Pest Control 1000ml – Permethrin 2.5 EC</t>
+          <t>Zero In Turbo Stream Pest Control 500ml – Permethrin 2.5 EC</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-092</t>
+          <t>MRT-WB-MTSGARDNING-091</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -1866,11 +1868,11 @@
         </is>
       </c>
       <c r="E23" s="11" t="n">
-        <v>1972</v>
+        <v>1109.25</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-128</t>
+          <t>MRT-WB-MTSGARDNING-127</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -1879,7 +1881,7 @@
         </is>
       </c>
       <c r="H23" s="11" t="n">
-        <v>1972</v>
+        <v>1109.25</v>
       </c>
       <c r="I23" s="11" t="n">
         <v>0</v>
@@ -1901,12 +1903,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Dark Knight Cockroach Killer 100ml – V-P 80% EC Pest Control</t>
+          <t>Zero In Turbo Stream Pest Control 1000ml – Permethrin 2.5 EC</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-093</t>
+          <t>MRT-WB-MTSGARDNING-092</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
@@ -1915,11 +1917,11 @@
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>3451</v>
+        <v>1972</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-129</t>
+          <t>MRT-WB-MTSGARDNING-128</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -1928,7 +1930,7 @@
         </is>
       </c>
       <c r="H24" s="11" t="n">
-        <v>3451</v>
+        <v>1972</v>
       </c>
       <c r="I24" s="11" t="n">
         <v>0</v>
@@ -1950,12 +1952,12 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Dark Knight Cockroach Killer 250ml – V-P 80% EC Pest Control</t>
+          <t>Dark Knight Cockroach Killer 100ml – V-P 80% EC Pest Control</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-094</t>
+          <t>MRT-WB-MTSGARDNING-093</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -1964,11 +1966,11 @@
         </is>
       </c>
       <c r="E25" s="11" t="n">
-        <v>554.625</v>
+        <v>3451</v>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-130</t>
+          <t>MRT-WB-MTSGARDNING-129</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -1977,7 +1979,7 @@
         </is>
       </c>
       <c r="H25" s="11" t="n">
-        <v>554.625</v>
+        <v>3451</v>
       </c>
       <c r="I25" s="11" t="n">
         <v>0</v>
@@ -1999,12 +2001,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Dark Knight Cockroach Killer 500ml – V-P 80% EC Pest Control</t>
+          <t>Dark Knight Cockroach Killer 250ml – V-P 80% EC Pest Control</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-095</t>
+          <t>MRT-WB-MTSGARDNING-094</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
@@ -2013,11 +2015,11 @@
         </is>
       </c>
       <c r="E26" s="11" t="n">
-        <v>1109.25</v>
+        <v>554.625</v>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-131</t>
+          <t>MRT-WB-MTSGARDNING-130</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -2026,7 +2028,7 @@
         </is>
       </c>
       <c r="H26" s="11" t="n">
-        <v>1109.25</v>
+        <v>554.625</v>
       </c>
       <c r="I26" s="11" t="n">
         <v>0</v>
@@ -2048,12 +2050,12 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Dark Knight Cockroach Killer 1000ml – V-P 80% EC Pest Control</t>
+          <t>Dark Knight Cockroach Killer 500ml – V-P 80% EC Pest Control</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-096</t>
+          <t>MRT-WB-MTSGARDNING-095</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
@@ -2062,11 +2064,11 @@
         </is>
       </c>
       <c r="E27" s="11" t="n">
-        <v>1972</v>
+        <v>1109.25</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>MRT-WB-MTSGARDNING-132</t>
+          <t>MRT-WB-MTSGARDNING-131</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
@@ -2075,7 +2077,7 @@
         </is>
       </c>
       <c r="H27" s="11" t="n">
-        <v>1972</v>
+        <v>1109.25</v>
       </c>
       <c r="I27" s="11" t="n">
         <v>0</v>
@@ -2086,6 +2088,55 @@
         </is>
       </c>
       <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>Drafted in store. Client must confirm if secondary listing is needed and which price is valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Dark Knight Cockroach Killer 1000ml – V-P 80% EC Pest Control</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>MRT-WB-MTSGARDNING-096</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Pest Control &gt; Roaches Control</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>1972</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>MRT-WB-MTSGARDNING-132</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Pest Control &gt; General Insects</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="n">
+        <v>1972</v>
+      </c>
+      <c r="I28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>Identical photos (2 files)</t>
+        </is>
+      </c>
+      <c r="K28" s="10" t="inlineStr">
         <is>
           <t>Drafted in store. Client must confirm if secondary listing is needed and which price is valid.</t>
         </is>
@@ -24803,67 +24854,67 @@
       </c>
     </row>
     <row r="343">
-      <c r="A343" s="15" t="n">
+      <c r="A343" s="19" t="n">
         <v>342</v>
       </c>
-      <c r="B343" s="15" t="inlineStr">
+      <c r="B343" s="20" t="inlineStr">
         <is>
           <t>MRT-WB-MTSGARDNING-060</t>
         </is>
       </c>
-      <c r="C343" s="15" t="inlineStr">
+      <c r="C343" s="19" t="inlineStr">
         <is>
           <t>MTS Gardening</t>
         </is>
       </c>
-      <c r="D343" s="16" t="inlineStr">
+      <c r="D343" s="21" t="inlineStr">
         <is>
           <t>Bromoxynil MCPA Herbicide 100ml – Broadleaf Weed Control</t>
         </is>
       </c>
-      <c r="E343" s="16" t="inlineStr">
+      <c r="E343" s="21" t="inlineStr">
         <is>
           <t>Gardening</t>
         </is>
       </c>
-      <c r="F343" s="16" t="inlineStr">
+      <c r="F343" s="21" t="inlineStr">
         <is>
           <t>Plants Insecticide/Fungicide</t>
         </is>
       </c>
-      <c r="G343" s="16" t="inlineStr">
+      <c r="G343" s="21" t="inlineStr">
         <is>
           <t>Plants Insecticide/Fungicide</t>
         </is>
       </c>
-      <c r="H343" s="17" t="n">
+      <c r="H343" s="22" t="n">
         <v>3451</v>
       </c>
-      <c r="I343" s="17" t="n">
+      <c r="I343" s="22" t="n">
         <v>4486</v>
       </c>
-      <c r="J343" s="15" t="inlineStr">
+      <c r="J343" s="19" t="inlineStr">
         <is>
           <t>+30%</t>
         </is>
       </c>
-      <c r="K343" s="18" t="n">
+      <c r="K343" s="23" t="n">
         <v>130</v>
       </c>
-      <c r="L343" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="M343" s="16" t="n">
+      <c r="L343" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="M343" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="N343" s="15" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="O343" s="16" t="inlineStr">
-        <is>
-          <t>Ready / Active</t>
+      <c r="N343" s="20" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="O343" s="21" t="inlineStr">
+        <is>
+          <t>Drafted: Duplicate listing of MRT-WB-MTSGARDNING-033</t>
         </is>
       </c>
     </row>

</xml_diff>